<commit_message>
Updates from building and debugging.
git-svn-id: http://10.105.1.46/svn/CCRT/Ccrt/branches/Common3700@26018 80089e14-fa6c-c64e-badd-1f0333e23b03
</commit_message>
<xml_diff>
--- a/Source/Tesla/Documentation/Tesla Host Interface Protocol.xlsx
+++ b/Source/Tesla/Documentation/Tesla Host Interface Protocol.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="16925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="17329"/>
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12795" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12795" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Port Setup" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="64">
   <si>
     <t>Hardware Protocol</t>
   </si>
@@ -199,13 +199,25 @@
     <t>RR Max Force</t>
   </si>
   <si>
-    <t>lbf x 11</t>
-  </si>
-  <si>
     <t>0x4D - Send Force Measurement</t>
   </si>
   <si>
     <t>0x50 - Periodic Message</t>
+  </si>
+  <si>
+    <t>Test Cycle Control</t>
+  </si>
+  <si>
+    <t>0x43 - Test Cycle Control</t>
+  </si>
+  <si>
+    <t>Test Cycle Control Type</t>
+  </si>
+  <si>
+    <t>0x42 - Begin Test Cycle</t>
+  </si>
+  <si>
+    <t>0x45 - End Test Cycle</t>
   </si>
 </sst>
 </file>
@@ -243,7 +255,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -331,11 +343,91 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0070C0"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF0070C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF0070C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF0070C0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF0070C0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0070C0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF0070C0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF0070C0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF0070C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF0070C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF0070C0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF0070C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -377,6 +469,26 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -799,7 +911,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>18</v>
@@ -947,7 +1059,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
@@ -1213,21 +1325,18 @@
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
       <c r="B14" s="12">
-        <f>B13+C13</f>
         <v>2</v>
       </c>
       <c r="C14" s="12">
         <v>1</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>18</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E14" s="12"/>
       <c r="F14" s="13"/>
       <c r="G14" s="12">
-        <f t="shared" ref="G14:G15" si="0">G13+H13</f>
+        <f>G13+H13</f>
         <v>2</v>
       </c>
       <c r="H14" s="12">
@@ -1241,153 +1350,147 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="16">
-        <f t="shared" si="0"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="12">
+        <f t="shared" ref="G15" si="0">G14+H14</f>
         <v>3</v>
       </c>
-      <c r="H15" s="16">
-        <v>1</v>
-      </c>
-      <c r="I15" s="17" t="s">
+      <c r="H15" s="12">
+        <v>1</v>
+      </c>
+      <c r="I15" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="J15" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="J15" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="12"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="14"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="16">
+        <v>3</v>
+      </c>
+      <c r="C17" s="16">
+        <v>1</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="17"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="18"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="8">
+      <c r="B20" s="8">
         <v>0</v>
       </c>
-      <c r="C18" s="8">
-        <v>1</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="C20" s="8">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="9"/>
-      <c r="G18" s="8">
+      <c r="E20" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="9"/>
+      <c r="G20" s="8">
         <v>0</v>
       </c>
-      <c r="H18" s="8">
-        <v>1</v>
-      </c>
-      <c r="I18" s="9" t="s">
+      <c r="H20" s="8">
+        <v>1</v>
+      </c>
+      <c r="I20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J18" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="11"/>
-      <c r="B19" s="12">
-        <f>B18+C18</f>
-        <v>1</v>
-      </c>
-      <c r="C19" s="12">
-        <v>1</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E19" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="13"/>
-      <c r="G19" s="12">
-        <f>G18+H18</f>
-        <v>1</v>
-      </c>
-      <c r="H19" s="2">
-        <v>1</v>
-      </c>
-      <c r="I19" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="J19" s="14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="11"/>
-      <c r="B20" s="12">
-        <f>B19+C19</f>
-        <v>2</v>
-      </c>
-      <c r="C20" s="12">
-        <v>1</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F20" s="13"/>
-      <c r="G20" s="12">
-        <f t="shared" ref="G20:G24" si="1">G19+H19</f>
-        <v>2</v>
-      </c>
-      <c r="H20" s="12">
-        <v>2</v>
-      </c>
-      <c r="I20" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>24</v>
+      <c r="J20" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="12"/>
+      <c r="B21" s="12">
+        <f>B20+C20</f>
+        <v>1</v>
+      </c>
+      <c r="C21" s="12">
+        <v>1</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>18</v>
+      </c>
       <c r="F21" s="13"/>
       <c r="G21" s="12">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="H21" s="12">
-        <v>2</v>
-      </c>
-      <c r="I21" s="13" t="s">
-        <v>39</v>
+        <f>G20+H20</f>
+        <v>1</v>
+      </c>
+      <c r="H21" s="2">
+        <v>1</v>
+      </c>
+      <c r="I21" s="19" t="s">
+        <v>57</v>
       </c>
       <c r="J21" s="14" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="12"/>
+      <c r="B22" s="12">
+        <f>B21+C21</f>
+        <v>2</v>
+      </c>
+      <c r="C22" s="12">
+        <v>1</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>18</v>
+      </c>
       <c r="F22" s="13"/>
       <c r="G22" s="12">
-        <f t="shared" si="1"/>
-        <v>6</v>
+        <f t="shared" ref="G22:G26" si="1">G21+H21</f>
+        <v>2</v>
       </c>
       <c r="H22" s="12">
         <v>2</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J22" s="14" t="s">
         <v>24</v>
@@ -1397,389 +1500,405 @@
       <c r="A23" s="11"/>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
-      <c r="D23" s="13"/>
+      <c r="D23" s="13" t="s">
+        <v>34</v>
+      </c>
       <c r="E23" s="12"/>
       <c r="F23" s="13"/>
       <c r="G23" s="12">
         <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="H23" s="12">
+        <v>2</v>
+      </c>
+      <c r="I23" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="12"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="12">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="H24" s="12">
+        <v>2</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="11"/>
+      <c r="B25" s="12">
+        <v>3</v>
+      </c>
+      <c r="C25" s="12">
+        <v>1</v>
+      </c>
+      <c r="D25" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" s="13"/>
+      <c r="G25" s="12">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="H23" s="12">
-        <v>2</v>
-      </c>
-      <c r="I23" s="13" t="s">
+      <c r="H25" s="12">
+        <v>2</v>
+      </c>
+      <c r="I25" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="J23" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="16">
+      <c r="J25" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="15"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="16">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="H24" s="16">
-        <v>1</v>
-      </c>
-      <c r="I24" s="17" t="s">
+      <c r="H26" s="16">
+        <v>1</v>
+      </c>
+      <c r="I26" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J24" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="J26" s="18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="8">
+      <c r="B29" s="8">
         <v>0</v>
       </c>
-      <c r="C27" s="8">
-        <v>1</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="C29" s="8">
+        <v>1</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E27" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F27" s="9"/>
-      <c r="G27" s="8">
+      <c r="E29" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="9"/>
+      <c r="G29" s="8">
         <v>0</v>
       </c>
-      <c r="H27" s="8">
-        <v>1</v>
-      </c>
-      <c r="I27" s="9" t="s">
+      <c r="H29" s="8">
+        <v>1</v>
+      </c>
+      <c r="I29" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J27" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="11"/>
-      <c r="B28" s="12">
-        <f>B27+C27</f>
-        <v>1</v>
-      </c>
-      <c r="C28" s="12">
-        <v>1</v>
-      </c>
-      <c r="D28" s="13" t="s">
+      <c r="J29" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="11"/>
+      <c r="B30" s="12">
+        <f>B29+C29</f>
+        <v>1</v>
+      </c>
+      <c r="C30" s="12">
+        <v>1</v>
+      </c>
+      <c r="D30" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="E28" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28" s="13"/>
-      <c r="G28" s="12">
-        <f>G27+H27</f>
-        <v>1</v>
-      </c>
-      <c r="H28" s="12">
-        <v>1</v>
-      </c>
-      <c r="I28" s="13" t="s">
+      <c r="E30" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="13"/>
+      <c r="G30" s="12">
+        <f>G29+H29</f>
+        <v>1</v>
+      </c>
+      <c r="H30" s="12">
+        <v>1</v>
+      </c>
+      <c r="I30" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="J28" s="14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="11"/>
-      <c r="B29" s="12">
-        <f>B28+C28</f>
-        <v>2</v>
-      </c>
-      <c r="C29" s="12">
-        <v>1</v>
-      </c>
-      <c r="D29" s="13" t="s">
+      <c r="J30" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="11"/>
+      <c r="B31" s="12">
+        <f>B30+C30</f>
+        <v>2</v>
+      </c>
+      <c r="C31" s="12">
+        <v>1</v>
+      </c>
+      <c r="D31" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F29" s="13"/>
-      <c r="G29" s="12">
-        <f t="shared" ref="G29:G30" si="2">G28+H28</f>
-        <v>2</v>
-      </c>
-      <c r="H29" s="12">
-        <v>1</v>
-      </c>
-      <c r="I29" s="13" t="s">
+      <c r="E31" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="13"/>
+      <c r="G31" s="12">
+        <f t="shared" ref="G31:G32" si="2">G30+H30</f>
+        <v>2</v>
+      </c>
+      <c r="H31" s="12">
+        <v>1</v>
+      </c>
+      <c r="I31" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="J29" s="14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="16">
+      <c r="J31" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="15"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="16">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="H30" s="16">
-        <v>1</v>
-      </c>
-      <c r="I30" s="17" t="s">
+      <c r="H32" s="16">
+        <v>1</v>
+      </c>
+      <c r="I32" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J30" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
+      <c r="J32" s="18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="8">
+      <c r="B35" s="8">
         <v>0</v>
       </c>
-      <c r="C33" s="8">
-        <v>1</v>
-      </c>
-      <c r="D33" s="9" t="s">
+      <c r="C35" s="8">
+        <v>1</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F33" s="9"/>
-      <c r="G33" s="8">
+      <c r="E35" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="9"/>
+      <c r="G35" s="8">
         <v>0</v>
       </c>
-      <c r="H33" s="8">
-        <v>1</v>
-      </c>
-      <c r="I33" s="9" t="s">
+      <c r="H35" s="8">
+        <v>1</v>
+      </c>
+      <c r="I35" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J33" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34" s="11"/>
-      <c r="B34" s="12">
-        <f>B33+C33</f>
-        <v>1</v>
-      </c>
-      <c r="C34" s="12">
-        <v>1</v>
-      </c>
-      <c r="D34" s="13" t="s">
+      <c r="J35" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="11"/>
+      <c r="B36" s="12">
+        <f>B35+C35</f>
+        <v>1</v>
+      </c>
+      <c r="C36" s="12">
+        <v>1</v>
+      </c>
+      <c r="D36" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F34" s="13"/>
-      <c r="G34" s="12">
-        <f>G33+H33</f>
-        <v>1</v>
-      </c>
-      <c r="H34" s="12">
-        <v>1</v>
-      </c>
-      <c r="I34" s="13" t="s">
+      <c r="E36" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="13"/>
+      <c r="G36" s="12">
+        <f>G35+H35</f>
+        <v>1</v>
+      </c>
+      <c r="H36" s="12">
+        <v>1</v>
+      </c>
+      <c r="I36" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="J34" s="14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35" s="11"/>
-      <c r="B35" s="12">
-        <f>B34+C34</f>
-        <v>2</v>
-      </c>
-      <c r="C35" s="12">
-        <v>1</v>
-      </c>
-      <c r="D35" s="13" t="s">
+      <c r="J36" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="11"/>
+      <c r="B37" s="12">
+        <f>B36+C36</f>
+        <v>2</v>
+      </c>
+      <c r="C37" s="12">
+        <v>1</v>
+      </c>
+      <c r="D37" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E35" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F35" s="13"/>
-      <c r="G35" s="12">
-        <f t="shared" ref="G35:G36" si="3">G34+H34</f>
-        <v>2</v>
-      </c>
-      <c r="H35" s="12">
-        <v>1</v>
-      </c>
-      <c r="I35" s="13" t="s">
+      <c r="E37" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="13"/>
+      <c r="G37" s="12">
+        <f t="shared" ref="G37:G38" si="3">G36+H36</f>
+        <v>2</v>
+      </c>
+      <c r="H37" s="12">
+        <v>1</v>
+      </c>
+      <c r="I37" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="J35" s="14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="17"/>
-      <c r="G36" s="16">
+      <c r="J37" s="14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="15"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="16">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="H36" s="16">
-        <v>1</v>
-      </c>
-      <c r="I36" s="17" t="s">
+      <c r="H38" s="16">
+        <v>1</v>
+      </c>
+      <c r="I38" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J36" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" s="7" t="s">
+      <c r="J38" s="18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B39" s="8">
+      <c r="B41" s="8">
         <v>0</v>
       </c>
-      <c r="C39" s="8">
-        <v>1</v>
-      </c>
-      <c r="D39" s="9" t="s">
+      <c r="C41" s="8">
+        <v>1</v>
+      </c>
+      <c r="D41" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E39" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F39" s="9"/>
-      <c r="G39" s="8">
+      <c r="E41" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F41" s="9"/>
+      <c r="G41" s="8">
         <v>0</v>
       </c>
-      <c r="H39" s="8">
-        <v>1</v>
-      </c>
-      <c r="I39" s="9" t="s">
+      <c r="H41" s="8">
+        <v>1</v>
+      </c>
+      <c r="I41" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="J39" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" s="11"/>
-      <c r="B40" s="12">
-        <f>B39+C39</f>
-        <v>1</v>
-      </c>
-      <c r="C40" s="12">
-        <v>1</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="E40" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F40" s="13"/>
-      <c r="G40" s="12">
-        <f>G39+H39</f>
-        <v>1</v>
-      </c>
-      <c r="H40" s="12">
-        <v>1</v>
-      </c>
-      <c r="I40" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J40" s="14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41" s="11"/>
-      <c r="B41" s="12">
-        <f>B40+C40</f>
-        <v>2</v>
-      </c>
-      <c r="C41" s="12">
-        <v>1</v>
-      </c>
-      <c r="D41" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="E41" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F41" s="13"/>
-      <c r="G41" s="12">
-        <f t="shared" ref="G41:G49" si="4">G40+H40</f>
-        <v>2</v>
-      </c>
-      <c r="H41" s="12">
-        <v>2</v>
-      </c>
-      <c r="I41" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="J41" s="14" t="s">
-        <v>24</v>
+      <c r="J41" s="10" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="11"/>
+      <c r="B42" s="12">
+        <f>B41+C41</f>
+        <v>1</v>
+      </c>
+      <c r="C42" s="12">
+        <v>1</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>18</v>
+      </c>
       <c r="F42" s="13"/>
       <c r="G42" s="12">
-        <f t="shared" si="4"/>
-        <v>4</v>
+        <f>G41+H41</f>
+        <v>1</v>
       </c>
       <c r="H42" s="12">
-        <v>2</v>
-      </c>
-      <c r="I42" s="19" t="s">
-        <v>50</v>
+        <v>1</v>
+      </c>
+      <c r="I42" s="13" t="s">
+        <v>48</v>
       </c>
       <c r="J42" s="14" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="11"/>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="12"/>
+      <c r="B43" s="12">
+        <f>B42+C42</f>
+        <v>2</v>
+      </c>
+      <c r="C43" s="12">
+        <v>1</v>
+      </c>
+      <c r="D43" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>18</v>
+      </c>
       <c r="F43" s="13"/>
       <c r="G43" s="12">
-        <f t="shared" si="4"/>
-        <v>6</v>
+        <f t="shared" ref="G43:G51" si="4">G42+H42</f>
+        <v>2</v>
       </c>
       <c r="H43" s="12">
         <v>2</v>
       </c>
-      <c r="I43" s="19" t="s">
-        <v>51</v>
+      <c r="I43" s="13" t="s">
+        <v>49</v>
       </c>
       <c r="J43" s="14" t="s">
         <v>24</v>
@@ -1787,20 +1906,16 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="11"/>
-      <c r="B44" s="12"/>
-      <c r="C44" s="12"/>
-      <c r="D44" s="13"/>
-      <c r="E44" s="12"/>
       <c r="F44" s="13"/>
       <c r="G44" s="12">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H44" s="12">
         <v>2</v>
       </c>
       <c r="I44" s="19" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="J44" s="14" t="s">
         <v>24</v>
@@ -1815,13 +1930,13 @@
       <c r="F45" s="13"/>
       <c r="G45" s="12">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H45" s="12">
         <v>2</v>
       </c>
       <c r="I45" s="19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J45" s="14" t="s">
         <v>24</v>
@@ -1836,13 +1951,13 @@
       <c r="F46" s="13"/>
       <c r="G46" s="12">
         <f t="shared" si="4"/>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H46" s="12">
         <v>2</v>
       </c>
       <c r="I46" s="19" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J46" s="14" t="s">
         <v>24</v>
@@ -1857,13 +1972,13 @@
       <c r="F47" s="13"/>
       <c r="G47" s="12">
         <f t="shared" si="4"/>
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H47" s="12">
         <v>2</v>
       </c>
       <c r="I47" s="19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J47" s="14" t="s">
         <v>24</v>
@@ -1878,49 +1993,233 @@
       <c r="F48" s="13"/>
       <c r="G48" s="12">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H48" s="12">
         <v>2</v>
       </c>
       <c r="I48" s="19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="J48" s="14" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49" s="15"/>
-      <c r="B49" s="16"/>
-      <c r="C49" s="16"/>
-      <c r="D49" s="17"/>
-      <c r="E49" s="16"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="16">
+      <c r="A49" s="11"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="12">
         <f t="shared" si="4"/>
-        <v>18</v>
-      </c>
-      <c r="H49" s="16">
-        <v>1</v>
-      </c>
-      <c r="I49" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H49" s="12">
+        <v>2</v>
+      </c>
+      <c r="I49" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="J49" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" s="11"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="13"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="12">
+        <f t="shared" si="4"/>
+        <v>16</v>
+      </c>
+      <c r="H50" s="12">
+        <v>2</v>
+      </c>
+      <c r="I50" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="J50" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" s="15"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="16"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="16">
+        <f t="shared" si="4"/>
+        <v>18</v>
+      </c>
+      <c r="H51" s="16">
+        <v>1</v>
+      </c>
+      <c r="I51" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="J49" s="18" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G50" s="12"/>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G51" s="12"/>
+      <c r="J51" s="18" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="G52" s="12"/>
     </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="B53" s="22">
+        <v>0</v>
+      </c>
+      <c r="C53" s="22">
+        <v>1</v>
+      </c>
+      <c r="D53" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F53" s="23"/>
+      <c r="G53" s="22">
+        <v>0</v>
+      </c>
+      <c r="H53" s="22">
+        <v>1</v>
+      </c>
+      <c r="I53" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="J53" s="24" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="25"/>
+      <c r="B54" s="12">
+        <f>B53+C53</f>
+        <v>1</v>
+      </c>
+      <c r="C54" s="12">
+        <v>1</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E54" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F54" s="13"/>
+      <c r="G54" s="12">
+        <f>G53+H53</f>
+        <v>1</v>
+      </c>
+      <c r="H54" s="12">
+        <v>1</v>
+      </c>
+      <c r="I54" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="J54" s="26" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="25"/>
+      <c r="B55" s="12">
+        <f>B54+C54</f>
+        <v>2</v>
+      </c>
+      <c r="C55" s="12">
+        <v>1</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F55" s="13"/>
+      <c r="G55" s="12">
+        <f t="shared" ref="G55:G56" si="5">G54+H54</f>
+        <v>2</v>
+      </c>
+      <c r="H55" s="12">
+        <v>1</v>
+      </c>
+      <c r="I55" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="J55" s="26" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="25"/>
+      <c r="B56" s="12"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E56" s="12"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="12">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="H56" s="12">
+        <v>1</v>
+      </c>
+      <c r="I56" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J56" s="26" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" s="25"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="E57" s="12"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="12"/>
+      <c r="I57" s="13"/>
+      <c r="J57" s="26"/>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="27"/>
+      <c r="B58" s="28">
+        <v>3</v>
+      </c>
+      <c r="C58" s="28">
+        <v>1</v>
+      </c>
+      <c r="D58" s="29" t="s">
+        <v>25</v>
+      </c>
+      <c r="E58" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="F58" s="29"/>
+      <c r="G58" s="28"/>
+      <c r="H58" s="28"/>
+      <c r="I58" s="29"/>
+      <c r="J58" s="30"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>